<commit_message>
test: add mock faker determinism guard
Refs: TASK-FK.3
</commit_message>
<xml_diff>
--- a/mock_data/bank_transactions.xlsx
+++ b/mock_data/bank_transactions.xlsx
@@ -611,7 +611,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>六盘水银行海门分行</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>招商银行上海分行</t>
+          <t>邯郸银行合肥分行</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>哈尔滨银行太原分行</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>建设银行杭州分行</t>
+          <t>石家庄银行惠州分行</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>北镇银行齐齐哈尔分行</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>工商银行上海分行</t>
+          <t>马鞍山银行淮安分行</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>贵阳银行南京分行</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>交通银行南京分行</t>
+          <t>马鞍山银行杭州分行</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>香港银行乌鲁木齐分行</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>农业银行苏州分行</t>
+          <t>通辽银行荆门分行</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>阜新银行郑州分行</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>浦发银行上海分行</t>
+          <t>哈尔滨银行石家庄分行</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>辽阳银行阜新分行</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>兰州银行深圳分行</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>石家庄银行长春分行</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1700,7 +1700,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>江苏银行无锡分行</t>
+          <t>石家庄银行西宁分行</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>拉萨银行南京分行</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>招商银行上海分行</t>
+          <t>淮安银行合山分行</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>梧州银行银川分行</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>宁波银行总行营业部</t>
+          <t>天津银行西宁分行</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">

</xml_diff>

<commit_message>
test: add mock batch structure guards
Refs: TASK-FK.4
</commit_message>
<xml_diff>
--- a/mock_data/bank_transactions.xlsx
+++ b/mock_data/bank_transactions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,27 +576,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>F1001</t>
+          <t>F10001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B202605210001</t>
+          <t>B202606000001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>09:10:00</t>
+          <t>10:07:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>六盘水银行海门分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -630,23 +630,23 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>100</v>
+        <v>97.34999999999999</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>100</v>
+        <v>97.34999999999999</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>10100</v>
+        <v>10197.35</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-21 09:10:00</t>
+          <t>2026-06-02 10:07:00</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -661,17 +661,17 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>6214********1001</t>
+          <t>6214********3001</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>上海云杉科技有限公司</t>
+          <t>恩悌网络有限公司</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>邯郸银行合肥分行</t>
+          <t>太原银行石家庄分行</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>网银转账</t>
+          <t>支付本月采购货款</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -716,34 +716,34 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>F1002</t>
+          <t>F10002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B202605210002</t>
+          <t>B202606000002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10:20:00</t>
+          <t>11:14:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>哈尔滨银行太原分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -777,23 +777,23 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>250.5</v>
+        <v>114.7</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>250.5</v>
+        <v>114.7</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>10350.5</v>
+        <v>10314.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-21 10:20:00</t>
+          <t>2026-06-03 11:14:00</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -808,32 +808,32 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>6214********1002</t>
+          <t>6214********3002</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>杭州青禾商贸有限公司</t>
+          <t>易动力信息有限公司</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>石家庄银行惠州分行</t>
+          <t>通辽银行荆门分行</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>柜面</t>
+          <t>手机银行</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>柜面入账</t>
+          <t>小王那笔材料钱</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>服务费</t>
+          <t>货款</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>TELLER_021</t>
+          <t>M_BANK</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -858,39 +858,39 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>CORE_COUNTER</t>
+          <t>MOBILE_BANKING</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>F1003</t>
+          <t>F10003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B202605210003</t>
+          <t>B202606000003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>11:30:00</t>
+          <t>12:21:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>北镇银行齐齐哈尔分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BATCH_PAYROLL</t>
+          <t>TRANSFER_OUT</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -924,10 +924,10 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>88.8</v>
+        <v>132.05</v>
       </c>
       <c r="M4" t="n">
-        <v>88.8</v>
+        <v>132.05</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -936,11 +936,11 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>10261.7</v>
+        <v>10167.95</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-05-21 11:30:00</t>
+          <t>2026-06-04 12:21:00</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -955,32 +955,32 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>6214********1003</t>
+          <t>6214********3003</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>员工代发虚拟户</t>
+          <t>佳禾科技有限公司</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>马鞍山银行淮安分行</t>
+          <t>长春银行石家庄分行</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>批量系统</t>
+          <t>网上银行</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>批量代发</t>
+          <t>支付物流运输费用</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>代发工资</t>
+          <t>费用</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -995,49 +995,49 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>BATCH_SYS</t>
+          <t>E_BANK</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>BATCH_PAY</t>
+          <t>TRF_OUT</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>BATCH_PAYMENT</t>
+          <t>E_BANKING</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>F1004</t>
+          <t>F10004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B202605210004</t>
+          <t>B202606000004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>13:40:00</t>
+          <t>13:28:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>贵阳银行南京分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1071,23 +1071,23 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>300</v>
+        <v>149.4</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>300</v>
+        <v>149.4</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>10561.7</v>
+        <v>10549.4</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-05-21 13:40:00</t>
+          <t>2026-06-05 13:28:00</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1102,27 +1102,27 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>6214********1004</t>
+          <t>6214********3004</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>南京北辰供应链有限公司</t>
+          <t>兰金电子网络有限公司</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>马鞍山银行杭州分行</t>
+          <t>哈尔滨银行淮安分行</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>清算平台</t>
+          <t>手机银行</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>清算金额差异</t>
+          <t>供应商催的那笔</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>CLEARING_SYS</t>
+          <t>M_BANK</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1152,39 +1152,39 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>CLEARING_PLATFORM</t>
+          <t>MOBILE_BANKING</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>金额差错样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>F1005</t>
+          <t>F10005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B202605210005</t>
+          <t>B202606000005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>15:00:00</t>
+          <t>14:35:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>香港银行乌鲁木齐分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1218,23 +1218,23 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>120</v>
+        <v>166.75</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>120</v>
+        <v>166.75</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>10681.7</v>
+        <v>10666.75</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-05-21 15:00:00</t>
+          <t>2026-06-06 14:35:00</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1249,17 +1249,17 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>6214********1005</t>
+          <t>6214********3005</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>苏州东海制造有限公司</t>
+          <t>易动力网络有限公司</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>通辽银行荆门分行</t>
+          <t>长春银行哈尔滨分行</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1269,12 +1269,12 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>银行端单边账</t>
+          <t>收到客户合同款项</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>预收款</t>
+          <t>货款</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
@@ -1304,34 +1304,34 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>银行端存在清算端缺失</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>F1008</t>
+          <t>F10006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B202605210008</t>
+          <t>B202606000006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>17:05:00</t>
+          <t>15:42:00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>阜新银行郑州分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1365,10 +1365,10 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>35.2</v>
+        <v>184.1</v>
       </c>
       <c r="M7" t="n">
-        <v>35.2</v>
+        <v>184.1</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -1377,11 +1377,11 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>10646.5</v>
+        <v>10415.9</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-05-21 17:05:00</t>
+          <t>2026-06-07 15:42:00</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1396,32 +1396,32 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>6214********1008</t>
+          <t>6214********3006</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>上海浦江物流有限公司</t>
+          <t>联软科技有限公司</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>哈尔滨银行石家庄分行</t>
+          <t>拉萨银行汕尾分行</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>网上银行</t>
+          <t>手机银行</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>网银付款</t>
+          <t>门店今天的款补上</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>物流费</t>
+          <t>费用</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>E_BANK</t>
+          <t>M_BANK</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1446,39 +1446,39 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>E_BANKING</t>
+          <t>MOBILE_BANKING</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>F1009</t>
+          <t>F10007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B202605210009</t>
+          <t>B202606000007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>17:20:00</t>
+          <t>16:49:00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>辽阳银行阜新分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1503,32 +1503,32 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>FEE</t>
+          <t>TRANSFER_IN</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>DEBIT</t>
+          <t>CREDIT</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>2</v>
+        <v>201.45</v>
       </c>
       <c r="M8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>201.45</v>
       </c>
       <c r="O8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>10644.5</v>
+        <v>10901.45</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-05-21 17:20:00</t>
+          <t>2026-06-08 16:49:00</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1543,32 +1543,32 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6214********1009</t>
+          <t>6214********3007</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>清算服务费虚拟户</t>
+          <t>凌颖信息科技有限公司</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>兰州银行深圳分行</t>
+          <t>贵阳银行哈尔滨分行</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>清算平台</t>
+          <t>网上银行</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>手续费扣收</t>
+          <t>收到客户合同款项</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>渠道手续费</t>
+          <t>货款</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -1583,49 +1583,49 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>CLEARING_SYS</t>
+          <t>E_BANK</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FEE_DEBIT</t>
+          <t>TRF_IN</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>CLEARING_PLATFORM</t>
+          <t>E_BANKING</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>F1010</t>
+          <t>F10008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B202605210010</t>
+          <t>B202606000008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>17:45:00</t>
+          <t>09:56:00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>石家庄银行长春分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1659,23 +1659,23 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>510</v>
+        <v>218.8</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>510</v>
+        <v>218.8</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>11154.5</v>
+        <v>11018.8</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-05-21 17:45:00</t>
+          <t>2026-06-09 09:56:00</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1690,32 +1690,32 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>6214********1010</t>
+          <t>6214********3008</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>无锡云帆材料有限公司</t>
+          <t>思优网络有限公司</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>石家庄银行西宁分行</t>
+          <t>通辽银行齐齐哈尔分行</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>网上银行</t>
+          <t>手机银行</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>跨行转账收入</t>
+          <t>小王那笔材料钱</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>材料款</t>
+          <t>货款</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>E_BANK</t>
+          <t>M_BANK</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
@@ -1740,39 +1740,39 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>E_BANKING</t>
+          <t>MOBILE_BANKING</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>F1011</t>
+          <t>F10009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B202605210011</t>
+          <t>B202606000009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>18:05:00</t>
+          <t>10:03:00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>拉萨银行南京分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1797,32 +1797,32 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>REFUND</t>
+          <t>TRANSFER_OUT</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CREDIT</t>
+          <t>DEBIT</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>18.8</v>
+        <v>236.15</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>236.15</v>
       </c>
       <c r="N10" t="n">
-        <v>18.8</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>11173.3</v>
+        <v>10663.85</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2026-05-21 18:05:00</t>
+          <t>2026-06-10 10:03:00</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1837,32 +1837,32 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>6214********1011</t>
+          <t>6214********3009</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>上海云杉科技有限公司</t>
+          <t>国讯科技有限公司</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>淮安银行合山分行</t>
+          <t>潜江银行广州分行</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>清算平台</t>
+          <t>网上银行</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>退款入账</t>
+          <t>收到客户合同款项</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>订单退款</t>
+          <t>费用</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1877,49 +1877,49 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>CLEARING_SYS</t>
+          <t>E_BANK</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>REFUND_IN</t>
+          <t>TRF_OUT</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>CLEARING_PLATFORM</t>
+          <t>E_BANKING</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>F1007</t>
+          <t>F10010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B202605210007</t>
+          <t>B202606000010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>16:30:00</t>
+          <t>11:10:00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>梧州银行银川分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1953,93 +1953,1269 @@
         </is>
       </c>
       <c r="L11" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>11253.5</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:10:00</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>6214********3010</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>商软冠联科技有限公司</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>北镇银行宜都分行</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>手机银行</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>上周那单尾款到了</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>货款</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>M_BANK</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>MOBILE_BANKING</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>批次正常自动平账样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F10011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B202606000011</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>12:17:00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>270.85</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>270.85</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>11370.85</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:17:00</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>6214********3011</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>立信电子传媒有限公司</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>郑州银行石家庄分行</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>收到年度框架协议款</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>货款</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>批次正常自动平账样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>F10012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B202606000012</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>13:24:00</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>TRANSFER_OUT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>288.2</v>
+      </c>
+      <c r="M13" t="n">
+        <v>288.2</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>10911.8</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:24:00</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>6214********3012</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>东方峻景网络有限公司</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>银川银行昆明分行</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>手机银行</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>老客户回款一笔</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>费用</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>M_BANK</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>TRF_OUT</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>MOBILE_BANKING</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>批次正常自动平账样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>F12001</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B202606010001</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>128</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>128</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>10128</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2026-06-01 09:00:00</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>6214********2001</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>明腾信息有限公司</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>兴安盟银行重庆分行</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>收到客户合同款项</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>货款</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>批次自动平账哨兵样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F12003</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B202606010003</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>10:10:00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>300</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>300</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>10339.5</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2026-06-01 10:10:00</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>6214********2003</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>南京北辰供应链有限公司</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>沈阳银行大冶分行</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>清算平台</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>补付款</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>货款</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>CLEARING_SYS</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>CLEARING_PLATFORM</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>MVP-1 金额不一致样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>F12004</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>B202606010004</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>REFUND</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
         <v>66.59999999999999</v>
       </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
         <v>66.59999999999999</v>
       </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>10748.3</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>2026-05-21 16:30:00</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>6222********0001</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>上海晨星贸易有限公司</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>6214********1007</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>10406.1</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:20:00</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>6214********2004</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
         <is>
           <t>宁波星河电子有限公司</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>天津银行西宁分行</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>手机银行</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>正常转账</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>零星收款</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>昆明银行哈尔滨分行</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>清算平台</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>退款</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>订单退款</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
         <is>
           <t>POSTED</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t>SH001</t>
         </is>
       </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>M_BANK</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>CLEARING_SYS</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>REFUND_IN</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>CLEARING_PLATFORM</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>MVP-1 摘要客户名不一致样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>F12006</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>B202606010006</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>45</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>45</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>10451.1</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:10:00</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>6214********2006</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>苏州东海制造有限公司</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>广州银行太原分行</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>代收代付</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>预收款</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
         <is>
           <t>TRF_IN</t>
         </is>
       </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>MOBILE_BANKING</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>正常平账样例</t>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>MVP-1 银行有企业无样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>F12007</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>B202606010007</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>10651.09</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:00:00</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>6214********2007</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>杭州青禾商贸有限公司</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>武汉银行嘉禾分行</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>临时款项</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>服务费</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>MVP-1 疑似重复入账样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>F12008</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>B202606010008</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>15:02:00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>10851.08</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:02:00</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>6214********2008</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>杭州青禾商贸有限公司</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>拉萨银行南宁分行</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>报销</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>服务费</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>MVP-1 疑似重复入账样例</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage faker mock data (#12)
* docs(adr): stage-faker-mock-data architectural decisions

* chore: add faker dev dependency

Refs: TASK-FK.1

* feat: fakerize mock decorative fields

Refs: TASK-FK.2

* test: add mock faker determinism guard

Refs: TASK-FK.3

* docs(adr): revise stage-faker-mock-data decisions — rebuild around realistic batch

* feat: add mock narrative pools

Refs: TASK-FK.1

* feat: rebuild bank enterprise mock batch

Refs: TASK-FK.2

* feat: rebuild bank clearing mock batch

Refs: TASK-FK.3

* test: add mock batch structure guards

Refs: TASK-FK.4

* docs(adr): archive stage-faker-mock-data decisions

* docs(adr): drop stage-faker-mock-data scratchpad

---------

Co-authored-by: “camellia <“yunshenbuzhichu@gmail.com”>
</commit_message>
<xml_diff>
--- a/mock_data/bank_transactions.xlsx
+++ b/mock_data/bank_transactions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE11"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,27 +576,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>F1001</t>
+          <t>F10001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B202605210001</t>
+          <t>B202606000001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>09:10:00</t>
+          <t>10:07:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -630,23 +630,23 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>100</v>
+        <v>97.34999999999999</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>100</v>
+        <v>97.34999999999999</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>10100</v>
+        <v>10197.35</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-21 09:10:00</t>
+          <t>2026-06-02 10:07:00</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -661,17 +661,17 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>6214********1001</t>
+          <t>6214********3001</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>上海云杉科技有限公司</t>
+          <t>恩悌网络有限公司</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>招商银行上海分行</t>
+          <t>太原银行石家庄分行</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>网银转账</t>
+          <t>支付本月采购货款</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -716,34 +716,34 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>F1002</t>
+          <t>F10002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B202605210002</t>
+          <t>B202606000002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10:20:00</t>
+          <t>11:14:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -777,23 +777,23 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>250.5</v>
+        <v>114.7</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>250.5</v>
+        <v>114.7</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>10350.5</v>
+        <v>10314.7</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-21 10:20:00</t>
+          <t>2026-06-03 11:14:00</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -808,32 +808,32 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>6214********1002</t>
+          <t>6214********3002</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>杭州青禾商贸有限公司</t>
+          <t>易动力信息有限公司</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>建设银行杭州分行</t>
+          <t>通辽银行荆门分行</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>柜面</t>
+          <t>手机银行</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>柜面入账</t>
+          <t>小王那笔材料钱</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>服务费</t>
+          <t>货款</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>TELLER_021</t>
+          <t>M_BANK</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
@@ -858,39 +858,39 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>CORE_COUNTER</t>
+          <t>MOBILE_BANKING</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>F1003</t>
+          <t>F10003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B202605210003</t>
+          <t>B202606000003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>11:30:00</t>
+          <t>12:21:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>BATCH_PAYROLL</t>
+          <t>TRANSFER_OUT</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -924,10 +924,10 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>88.8</v>
+        <v>132.05</v>
       </c>
       <c r="M4" t="n">
-        <v>88.8</v>
+        <v>132.05</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
@@ -936,11 +936,11 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>10261.7</v>
+        <v>10167.95</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-05-21 11:30:00</t>
+          <t>2026-06-04 12:21:00</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -955,32 +955,32 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>6214********1003</t>
+          <t>6214********3003</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>员工代发虚拟户</t>
+          <t>佳禾科技有限公司</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>工商银行上海分行</t>
+          <t>长春银行石家庄分行</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>批量系统</t>
+          <t>网上银行</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>批量代发</t>
+          <t>支付物流运输费用</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>代发工资</t>
+          <t>费用</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -995,49 +995,49 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>BATCH_SYS</t>
+          <t>E_BANK</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>BATCH_PAY</t>
+          <t>TRF_OUT</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>BATCH_PAYMENT</t>
+          <t>E_BANKING</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>F1004</t>
+          <t>F10004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B202605210004</t>
+          <t>B202606000004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>13:40:00</t>
+          <t>13:28:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1071,23 +1071,23 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>300</v>
+        <v>149.4</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>300</v>
+        <v>149.4</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>10561.7</v>
+        <v>10549.4</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-05-21 13:40:00</t>
+          <t>2026-06-05 13:28:00</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1102,27 +1102,27 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>6214********1004</t>
+          <t>6214********3004</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>南京北辰供应链有限公司</t>
+          <t>兰金电子网络有限公司</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>交通银行南京分行</t>
+          <t>哈尔滨银行淮安分行</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>清算平台</t>
+          <t>手机银行</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>清算金额差异</t>
+          <t>供应商催的那笔</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>CLEARING_SYS</t>
+          <t>M_BANK</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
@@ -1152,39 +1152,39 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>CLEARING_PLATFORM</t>
+          <t>MOBILE_BANKING</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>金额差错样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>F1005</t>
+          <t>F10005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B202605210005</t>
+          <t>B202606000005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>15:00:00</t>
+          <t>14:35:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1218,23 +1218,23 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>120</v>
+        <v>166.75</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>120</v>
+        <v>166.75</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>10681.7</v>
+        <v>10666.75</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-05-21 15:00:00</t>
+          <t>2026-06-06 14:35:00</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1249,17 +1249,17 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>6214********1005</t>
+          <t>6214********3005</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>苏州东海制造有限公司</t>
+          <t>易动力网络有限公司</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>农业银行苏州分行</t>
+          <t>长春银行哈尔滨分行</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
@@ -1269,12 +1269,12 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>银行端单边账</t>
+          <t>收到客户合同款项</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>预收款</t>
+          <t>货款</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
@@ -1304,34 +1304,34 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>银行端存在清算端缺失</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>F1008</t>
+          <t>F10006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B202605210008</t>
+          <t>B202606000006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>17:05:00</t>
+          <t>15:42:00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1365,10 +1365,10 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>35.2</v>
+        <v>184.1</v>
       </c>
       <c r="M7" t="n">
-        <v>35.2</v>
+        <v>184.1</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -1377,11 +1377,11 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>10646.5</v>
+        <v>10415.9</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-05-21 17:05:00</t>
+          <t>2026-06-07 15:42:00</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1396,32 +1396,32 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>6214********1008</t>
+          <t>6214********3006</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>上海浦江物流有限公司</t>
+          <t>联软科技有限公司</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>浦发银行上海分行</t>
+          <t>拉萨银行汕尾分行</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>网上银行</t>
+          <t>手机银行</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>网银付款</t>
+          <t>门店今天的款补上</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>物流费</t>
+          <t>费用</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>E_BANK</t>
+          <t>M_BANK</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
@@ -1446,39 +1446,39 @@
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>E_BANKING</t>
+          <t>MOBILE_BANKING</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>F1009</t>
+          <t>F10007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B202605210009</t>
+          <t>B202606000007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>17:20:00</t>
+          <t>16:49:00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1503,32 +1503,32 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>FEE</t>
+          <t>TRANSFER_IN</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>DEBIT</t>
+          <t>CREDIT</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>2</v>
+        <v>201.45</v>
       </c>
       <c r="M8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0</v>
+        <v>201.45</v>
       </c>
       <c r="O8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>10644.5</v>
+        <v>10901.45</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-05-21 17:20:00</t>
+          <t>2026-06-08 16:49:00</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1543,32 +1543,32 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>6214********1009</t>
+          <t>6214********3007</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>清算服务费虚拟户</t>
+          <t>凌颖信息科技有限公司</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>贵阳银行哈尔滨分行</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>清算平台</t>
+          <t>网上银行</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>手续费扣收</t>
+          <t>收到客户合同款项</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>渠道手续费</t>
+          <t>货款</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -1583,49 +1583,49 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>CLEARING_SYS</t>
+          <t>E_BANK</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>FEE_DEBIT</t>
+          <t>TRF_IN</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>CLEARING_PLATFORM</t>
+          <t>E_BANKING</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>F1010</t>
+          <t>F10008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B202605210010</t>
+          <t>B202606000008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>17:45:00</t>
+          <t>09:56:00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1659,23 +1659,23 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>510</v>
+        <v>218.8</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>510</v>
+        <v>218.8</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>11154.5</v>
+        <v>11018.8</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-05-21 17:45:00</t>
+          <t>2026-06-09 09:56:00</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1690,32 +1690,32 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>6214********1010</t>
+          <t>6214********3008</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>无锡云帆材料有限公司</t>
+          <t>思优网络有限公司</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>江苏银行无锡分行</t>
+          <t>通辽银行齐齐哈尔分行</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>网上银行</t>
+          <t>手机银行</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>跨行转账收入</t>
+          <t>小王那笔材料钱</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>材料款</t>
+          <t>货款</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>E_BANK</t>
+          <t>M_BANK</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
@@ -1740,39 +1740,39 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>E_BANKING</t>
+          <t>MOBILE_BANKING</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>F1011</t>
+          <t>F10009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B202605210011</t>
+          <t>B202606000009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>18:05:00</t>
+          <t>10:03:00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1797,32 +1797,32 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>REFUND</t>
+          <t>TRANSFER_OUT</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CREDIT</t>
+          <t>DEBIT</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>18.8</v>
+        <v>236.15</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>236.15</v>
       </c>
       <c r="N10" t="n">
-        <v>18.8</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>11173.3</v>
+        <v>10663.85</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2026-05-21 18:05:00</t>
+          <t>2026-06-10 10:03:00</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1837,32 +1837,32 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>6214********1011</t>
+          <t>6214********3009</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>上海云杉科技有限公司</t>
+          <t>国讯科技有限公司</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>招商银行上海分行</t>
+          <t>潜江银行广州分行</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>清算平台</t>
+          <t>网上银行</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>退款入账</t>
+          <t>收到客户合同款项</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>订单退款</t>
+          <t>费用</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1877,49 +1877,49 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>CLEARING_SYS</t>
+          <t>E_BANK</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>REFUND_IN</t>
+          <t>TRF_OUT</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>CLEARING_PLATFORM</t>
+          <t>E_BANKING</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>正常平账样例</t>
+          <t>批次正常自动平账样例</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>F1007</t>
+          <t>F10010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B202605210007</t>
+          <t>B202606000010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>16:30:00</t>
+          <t>11:10:00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>中国银行上海分行</t>
+          <t>上海银行浦东分行</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1953,93 +1953,1269 @@
         </is>
       </c>
       <c r="L11" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>11253.5</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:10:00</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>6214********3010</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>商软冠联科技有限公司</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>北镇银行宜都分行</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>手机银行</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>上周那单尾款到了</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>货款</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>M_BANK</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>MOBILE_BANKING</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>批次正常自动平账样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F10011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B202606000011</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>12:17:00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>270.85</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>270.85</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>11370.85</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:17:00</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>6214********3011</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>立信电子传媒有限公司</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>郑州银行石家庄分行</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>收到年度框架协议款</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>货款</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>批次正常自动平账样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>F10012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B202606000012</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>13:24:00</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>TRANSFER_OUT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>DEBIT</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>288.2</v>
+      </c>
+      <c r="M13" t="n">
+        <v>288.2</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>10911.8</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:24:00</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>6214********3012</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>东方峻景网络有限公司</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>银川银行昆明分行</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>手机银行</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>老客户回款一笔</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>费用</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>M_BANK</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>TRF_OUT</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>MOBILE_BANKING</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>批次正常自动平账样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>F12001</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B202606010001</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>09:00:00</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>128</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>128</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>10128</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>2026-06-01 09:00:00</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>6214********2001</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>明腾信息有限公司</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>兴安盟银行重庆分行</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>收到客户合同款项</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>货款</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t>批次自动平账哨兵样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F12003</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B202606010003</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>10:10:00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>300</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>300</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>10339.5</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>2026-06-01 10:10:00</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>6214********2003</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>南京北辰供应链有限公司</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>沈阳银行大冶分行</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>清算平台</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>补付款</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>货款</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>CLEARING_SYS</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>CLEARING_PLATFORM</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>MVP-1 金额不一致样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>F12004</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>B202606010004</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>11:20:00</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>REFUND</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
         <v>66.59999999999999</v>
       </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
         <v>66.59999999999999</v>
       </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>10748.3</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>2026-05-21 16:30:00</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>6222********0001</t>
-        </is>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>上海晨星贸易有限公司</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>6214********1007</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="n">
+        <v>10406.1</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>2026-06-01 11:20:00</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>6214********2004</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
         <is>
           <t>宁波星河电子有限公司</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>宁波银行总行营业部</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>手机银行</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>正常转账</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>零星收款</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>昆明银行哈尔滨分行</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>清算平台</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>退款</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>订单退款</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
         <is>
           <t>POSTED</t>
         </is>
       </c>
-      <c r="AA11" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t>SH001</t>
         </is>
       </c>
-      <c r="AB11" t="inlineStr">
-        <is>
-          <t>M_BANK</t>
-        </is>
-      </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>CLEARING_SYS</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>REFUND_IN</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>CLEARING_PLATFORM</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>MVP-1 摘要客户名不一致样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>F12006</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>B202606010006</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>14:10:00</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>45</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>45</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>10451.1</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2026-06-01 14:10:00</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>6214********2006</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>苏州东海制造有限公司</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>广州银行太原分行</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>代收代付</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>预收款</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC17" t="inlineStr">
         <is>
           <t>TRF_IN</t>
         </is>
       </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>MOBILE_BANKING</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>正常平账样例</t>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr">
+        <is>
+          <t>MVP-1 银行有企业无样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>F12007</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>B202606010007</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>15:00:00</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="n">
+        <v>10651.09</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:00:00</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>6214********2007</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>杭州青禾商贸有限公司</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>武汉银行嘉禾分行</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>临时款项</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>服务费</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>MVP-1 疑似重复入账样例</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>F12008</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>B202606010008</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>15:02:00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>上海银行浦东分行</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>TRANSFER_IN</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>CREDIT</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>199.99</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="n">
+        <v>10851.08</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:02:00</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>6222********0001</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>上海晨星贸易有限公司</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>6214********2008</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>杭州青禾商贸有限公司</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>拉萨银行南宁分行</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>网上银行</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>报销</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>服务费</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>POSTED</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>SH001</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>E_BANK</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>TRF_IN</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>E_BANKING</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>MVP-1 疑似重复入账样例</t>
         </is>
       </c>
     </row>

</xml_diff>